<commit_message>
Update Natura 2000-linked empirical tables
</commit_message>
<xml_diff>
--- a/empirical/results/INNATURA_ASV_table_decontaminated.xlsx
+++ b/empirical/results/INNATURA_ASV_table_decontaminated.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="asv table" sheetId="1" r:id="R12415826d9ea4c98"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="asv table" sheetId="1" r:id="Rcb38084410a74fd2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -10,39 +10,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:si>
-    <x:t xml:space="preserve">Group</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Family</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Species</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">BAR</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">BIA</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">FRA</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">NOV</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">STA</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">CANA</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">MER</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">PET</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Birds</x:t>
   </x:si>
   <x:si>
@@ -152,9 +119,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Turdus philomelos</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Amplicon Sequence Variant (ASV) table generated from eDNA metabarcoding across eight sampling sites within N2K locations. Human sequences and potential contaminants have been excluded. Sample IDs denote N2K site IT1342806 “M. Verruga - M. Zenone Roccagrande - M. Pu” (VERR1–VERR5) and N2K site IT1343412 “Deiva - Bracco - Pietra di Vasca - Mola” (DEIV1–DEIV3).</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -561,12 +525,18 @@
     <x:xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="4">
+  <x:cellXfs count="6">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <x:xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <x:xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="42">
@@ -814,53 +784,68 @@
     <x:col min="1" max="1" width="10.44140625" customWidth="1"/>
     <x:col min="2" max="2" width="13.21875" customWidth="1"/>
     <x:col min="3" max="3" width="23.33203125" customWidth="1"/>
-    <x:col min="4" max="4" width="9" customWidth="1"/>
+    <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="18" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="18" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="18" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="18" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="18" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="2" t="s">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="B1" s="2" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C1" s="2" t="s">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="D1" s="3" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="E1" s="3" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="F1" s="3" t="s">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="G1" s="3" t="s">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="H1" s="3" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="I1" s="3" t="s">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="J1" s="3" t="s">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="K1" s="3" t="s">
-        <x:v>10</x:v>
+      <x:c r="A1" s="2" t="str">
+        <x:v>Group</x:v>
+      </x:c>
+      <x:c r="B1" s="2" t="str">
+        <x:v>Family</x:v>
+      </x:c>
+      <x:c r="C1" s="2" t="str">
+        <x:v>Species</x:v>
+      </x:c>
+      <x:c r="D1" s="4" t="str">
+        <x:v>BAR
+(IT1342806)</x:v>
+      </x:c>
+      <x:c r="E1" s="4" t="str">
+        <x:v>BIA
+(IT1342806)</x:v>
+      </x:c>
+      <x:c r="F1" s="4" t="str">
+        <x:v>FRA
+(IT1342806)</x:v>
+      </x:c>
+      <x:c r="G1" s="4" t="str">
+        <x:v>NOV
+(IT1342806)</x:v>
+      </x:c>
+      <x:c r="H1" s="4" t="str">
+        <x:v>STA
+(IT1342806)</x:v>
+      </x:c>
+      <x:c r="I1" s="4" t="str">
+        <x:v>CANA
+(IT1343412)</x:v>
+      </x:c>
+      <x:c r="J1" s="4" t="str">
+        <x:v>MER
+(IT1343412)</x:v>
+      </x:c>
+      <x:c r="K1" s="4" t="str">
+        <x:v>PET
+(IT1343412)</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
       <x:c r="A2" t="s">
-        <x:v>11</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="B2" t="s">
-        <x:v>12</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C2" s="1" t="s">
-        <x:v>13</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D2">
         <x:v>0</x:v>
@@ -889,13 +874,13 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" t="s">
-        <x:v>14</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="B3" t="s">
-        <x:v>15</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="C3" s="1" t="s">
-        <x:v>16</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="D3">
         <x:v>0</x:v>
@@ -924,13 +909,13 @@
     </x:row>
     <x:row r="4">
       <x:c r="A4" t="s">
-        <x:v>14</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="B4" t="s">
-        <x:v>17</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="C4" s="1" t="s">
-        <x:v>18</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="D4">
         <x:v>0</x:v>
@@ -959,13 +944,13 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" t="s">
-        <x:v>19</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="B5" t="s">
-        <x:v>20</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="C5" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="D5">
         <x:v>497</x:v>
@@ -994,13 +979,13 @@
     </x:row>
     <x:row r="6">
       <x:c r="A6" t="s">
-        <x:v>19</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="B6" t="s">
-        <x:v>20</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="C6" s="1" t="s">
-        <x:v>22</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="D6">
         <x:v>0</x:v>
@@ -1029,13 +1014,13 @@
     </x:row>
     <x:row r="7">
       <x:c r="A7" t="s">
-        <x:v>19</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="B7" t="s">
-        <x:v>20</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="C7" s="1" t="s">
-        <x:v>23</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="D7">
         <x:v>0</x:v>
@@ -1064,13 +1049,13 @@
     </x:row>
     <x:row r="8">
       <x:c r="A8" t="s">
-        <x:v>24</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="B8" t="s">
-        <x:v>25</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="C8" s="1" t="s">
-        <x:v>26</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="D8">
         <x:v>0</x:v>
@@ -1099,13 +1084,13 @@
     </x:row>
     <x:row r="9">
       <x:c r="A9" t="s">
-        <x:v>11</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="B9" t="s">
-        <x:v>27</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="C9" s="1" t="s">
-        <x:v>28</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="D9">
         <x:v>1162</x:v>
@@ -1134,13 +1119,13 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" t="s">
-        <x:v>11</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="B10" t="s">
-        <x:v>29</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="C10" s="1" t="s">
-        <x:v>30</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="D10">
         <x:v>13</x:v>
@@ -1169,13 +1154,13 @@
     </x:row>
     <x:row r="11">
       <x:c r="A11" t="s">
-        <x:v>11</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="B11" t="str">
         <x:v>Muscicapidae</x:v>
       </x:c>
       <x:c r="C11" s="1" t="s">
-        <x:v>31</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="D11">
         <x:v>0</x:v>
@@ -1204,13 +1189,13 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" t="s">
-        <x:v>24</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="B12" t="s">
-        <x:v>32</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="C12" s="1" t="s">
-        <x:v>33</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="D12">
         <x:v>0</x:v>
@@ -1242,10 +1227,10 @@
         <x:v>Fish</x:v>
       </x:c>
       <x:c r="B13" t="s">
-        <x:v>34</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="C13" s="1" t="s">
-        <x:v>35</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="D13">
         <x:v>923</x:v>
@@ -1274,13 +1259,13 @@
     </x:row>
     <x:row r="14">
       <x:c r="A14" t="s">
-        <x:v>11</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="B14" t="str">
         <x:v>Paridae</x:v>
       </x:c>
       <x:c r="C14" s="1" t="s">
-        <x:v>36</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="D14">
         <x:v>0</x:v>
@@ -1309,13 +1294,13 @@
     </x:row>
     <x:row r="15">
       <x:c r="A15" t="s">
-        <x:v>14</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="B15" t="s">
-        <x:v>17</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="C15" s="1" t="s">
-        <x:v>37</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="D15">
         <x:v>332</x:v>
@@ -1344,13 +1329,13 @@
     </x:row>
     <x:row r="16">
       <x:c r="A16" t="s">
-        <x:v>19</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="B16" t="s">
-        <x:v>38</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="C16" s="1" t="s">
-        <x:v>39</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="D16">
         <x:v>4118</x:v>
@@ -1379,13 +1364,13 @@
     </x:row>
     <x:row r="17">
       <x:c r="A17" t="s">
-        <x:v>14</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="B17" t="s">
-        <x:v>17</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="C17" s="1" t="s">
-        <x:v>40</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="D17">
         <x:v>0</x:v>
@@ -1414,13 +1399,13 @@
     </x:row>
     <x:row r="18">
       <x:c r="A18" t="s">
-        <x:v>19</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="B18" t="s">
-        <x:v>41</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C18" s="1" t="s">
-        <x:v>42</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="D18">
         <x:v>0</x:v>
@@ -1449,13 +1434,13 @@
     </x:row>
     <x:row r="19">
       <x:c r="A19" t="s">
-        <x:v>14</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="B19" t="s">
-        <x:v>34</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="C19" s="1" t="s">
-        <x:v>43</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="D19">
         <x:v>565</x:v>
@@ -1484,13 +1469,13 @@
     </x:row>
     <x:row r="20">
       <x:c r="A20" t="s">
-        <x:v>14</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="B20" t="s">
-        <x:v>34</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="C20" s="1" t="s">
-        <x:v>44</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="D20">
         <x:v>17972</x:v>
@@ -1519,13 +1504,13 @@
     </x:row>
     <x:row r="21">
       <x:c r="A21" t="s">
-        <x:v>14</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="B21" t="s">
-        <x:v>17</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="C21" s="1" t="s">
-        <x:v>45</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="D21">
         <x:v>345</x:v>
@@ -1554,13 +1539,13 @@
     </x:row>
     <x:row r="22">
       <x:c r="A22" t="s">
-        <x:v>11</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="B22" t="s">
-        <x:v>46</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="C22" s="1" t="s">
-        <x:v>47</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="D22">
         <x:v>0</x:v>
@@ -1587,12 +1572,25 @@
         <x:v>0</x:v>
       </x:c>
     </x:row>
-    <x:row r="24">
-      <x:c r="A24" t="s">
-        <x:v>48</x:v>
-      </x:c>
+    <x:row r="24" ht="32" customHeight="1">
+      <x:c r="A24" s="5" t="str">
+        <x:v>Decontaminated taxon read counts by sampling site. BAR, BIA, FRA, NOV and STA are within Natura 2000 site IT1342806; CANA, MER and PET are within Natura 2000 site IT1343412. Human sequences and potential contaminants have been excluded.</x:v>
+      </x:c>
+      <x:c r="B24" s="5"/>
+      <x:c r="C24" s="5"/>
+      <x:c r="D24" s="5"/>
+      <x:c r="E24" s="5"/>
+      <x:c r="F24" s="5"/>
+      <x:c r="G24" s="5"/>
+      <x:c r="H24" s="5"/>
+      <x:c r="I24" s="5"/>
+      <x:c r="J24" s="5"/>
+      <x:c r="K24" s="5"/>
     </x:row>
   </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A24:K24"/>
+  </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
</xml_diff>